<commit_message>
fix: verify dossier workbook printing and safe upload cleanup
</commit_message>
<xml_diff>
--- a/frontend/docs/reviews/dossiers-phase-three/dossier.xlsx
+++ b/frontend/docs/reviews/dossiers-phase-three/dossier.xlsx
@@ -63,15 +63,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="92">
   <si>
     <t>هوية الإضبارة · مشفى محمد بن زايد الإماراتي</t>
   </si>
   <si>
-    <t>رقم التقرير: DOS-19-2026-000004 | الإصدار: 2026-09-15 13:49:36 · Asia/Damascus</t>
-  </si>
-  <si>
-    <t>المنشأة: منشأة اختبار الخدمات | أصدره: Diego Sawayn DVM</t>
+    <t>رقم التقرير: DOS-37-2026-000004 | الإصدار: 2026-09-15 15:07:49 · Asia/Damascus</t>
+  </si>
+  <si>
+    <t>المنشأة: منشأة اختبار الخدمات | أصدره: Paris Lakin</t>
   </si>
   <si>
     <t>نطاق التقرير: تقرير فردي ضمن المنشأة المصرح بها</t>
@@ -89,15 +89,12 @@
     <t>كود الإضبارة</t>
   </si>
   <si>
-    <t>PH3-ellussbd-1440</t>
+    <t>PH3-ict6ccul-1440</t>
   </si>
   <si>
     <t>تاريخ فتح الإضبارة</t>
   </si>
   <si>
-    <t>2001-01-01</t>
-  </si>
-  <si>
     <t>المريض</t>
   </si>
   <si>
@@ -107,7 +104,7 @@
     <t>كود المريض</t>
   </si>
   <si>
-    <t>P-91960710-79ee-4c03-8afb-572f98af67b4</t>
+    <t>P-aebc68d7-ef77-46cc-9fe7-3af10bf3c878</t>
   </si>
   <si>
     <t>حالة الإضبارة</t>
@@ -119,7 +116,7 @@
     <t>آخر زيارة فعلية</t>
   </si>
   <si>
-    <t>V-37a700fa-e57d-4e41-9732-a62e2c87a11c · 2001-03-02 · مكتملة</t>
+    <t>V-40d7b2ca-6e2f-4a85-9a26-96902951b35a · 2001-03-02 · مكتملة</t>
   </si>
   <si>
     <t>بيانات المريض الحالية · مشفى محمد بن زايد الإماراتي</t>
@@ -200,16 +197,16 @@
     <t>التسلسل الزمني للزيارات · مشفى محمد بن زايد الإماراتي</t>
   </si>
   <si>
-    <t>رقم التقرير: DOS-19-2026-000004</t>
-  </si>
-  <si>
-    <t>الإصدار: 2026-09-15 13:49:36 · Asia/Damascus</t>
+    <t>رقم التقرير: DOS-37-2026-000004</t>
+  </si>
+  <si>
+    <t>الإصدار: 2026-09-15 15:07:49 · Asia/Damascus</t>
   </si>
   <si>
     <t>المنشأة: منشأة اختبار الخدمات</t>
   </si>
   <si>
-    <t>أصدره: Diego Sawayn DVM</t>
+    <t>أصدره: Paris Lakin</t>
   </si>
   <si>
     <t>نطاق التقرير: الأحدث أولًا حسب التاريخ الفعلي ثم معرّف الزيارة. الإحالة الواردة مستقلة عن النتيجة والإحالة الصادرة.</t>
@@ -227,7 +224,7 @@
     <t>الإحالة الواردة</t>
   </si>
   <si>
-    <t>V-37a700fa-e57d-4e41-9732-a62e2c87a11c</t>
+    <t>V-40d7b2ca-6e2f-4a85-9a26-96902951b35a</t>
   </si>
   <si>
     <t>مكتملة</t>
@@ -295,13 +292,13 @@
     <t>نطاق التقرير: وصفة فقط؛ لا تمثل صرفًا أو إعطاءً. تعريف الدواء محفوظ وقت إدراجه.</t>
   </si>
   <si>
-    <t>NEW-ellussbd-1440 · دواء جديد اصطناعي 1440 ellussbd</t>
+    <t>NEW-ict6ccul-1440 · دواء جديد اصطناعي 1440 ict6ccul</t>
   </si>
   <si>
     <t>تعليمات اصطناعية 1</t>
   </si>
   <si>
-    <t>RX-ellussbd · دواء اختبار ellussbd</t>
+    <t>RX-ict6ccul · دواء اختبار ict6ccul</t>
   </si>
   <si>
     <t>تعليمات اصطناعية 2</t>
@@ -344,17 +341,15 @@
   </si>
   <si>
     <t>sample.png</t>
-  </si>
-  <si>
-    <t>2026-09-15 10:49:27</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd hh:mm:ss"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -435,7 +430,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="84">
+  <cellXfs count="86">
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
     <xf xfId="0" fontId="1" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" shrinkToFit="false"/>
@@ -452,6 +447,9 @@
     <xf xfId="0" fontId="0" numFmtId="0" fillId="3" borderId="1" applyFont="0" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" shrinkToFit="false"/>
     </xf>
+    <xf xfId="0" fontId="0" numFmtId="164" fillId="3" borderId="1" applyFont="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" shrinkToFit="false"/>
+    </xf>
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
     <xf xfId="0" fontId="1" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" shrinkToFit="false"/>
@@ -662,6 +660,9 @@
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" shrinkToFit="false"/>
     </xf>
     <xf xfId="0" fontId="0" numFmtId="1" fillId="0" borderId="1" applyFont="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="0" numFmtId="165" fillId="0" borderId="1" applyFont="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" shrinkToFit="false"/>
     </xf>
   </cellXfs>
@@ -1446,40 +1447,40 @@
       <c r="A10" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="5" t="s">
-        <v>10</v>
+      <c r="B10" s="6">
+        <v>36892.0</v>
       </c>
     </row>
     <row r="11" spans="1:2" customHeight="1" ht="27.25">
       <c r="A11" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11" s="4" t="s">
         <v>11</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="12" spans="1:2" customHeight="1" ht="27.25">
       <c r="A12" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B12" s="5" t="s">
         <v>13</v>
-      </c>
-      <c r="B12" s="5" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="13" spans="1:2" customHeight="1" ht="27.25">
       <c r="A13" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B13" s="4" t="s">
         <v>15</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="14" spans="1:2" customHeight="1" ht="27.25">
       <c r="A14" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B14" s="5" t="s">
         <v>17</v>
-      </c>
-      <c r="B14" s="5" t="s">
-        <v>18</v>
       </c>
     </row>
   </sheetData>
@@ -1492,10 +1493,11 @@
     <mergeCell ref="A6:B6"/>
   </mergeCells>
   <printOptions gridLines="false" gridLinesSet="true"/>
-  <pageMargins left="0.47" right="0.47" top="0.35" bottom="0.5" header="0.3" footer="0.2"/>
+  <pageMargins left="0.47" right="0.47" top="0.5" bottom="0.5" header="0.18" footer="0.2"/>
   <pageSetup paperSize="9" orientation="portrait" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver"/>
   <headerFooter differentOddEven="false" differentFirst="false" scaleWithDoc="true" alignWithMargins="true">
-    <oddFooter>&amp;"Cairo,Regular"&amp;9&amp;CDOS-19-2026-000004 | &amp;P / &amp;N</oddFooter>
+    <oddHeader>&amp;R&amp;"Cairo,Regular"&amp;9هوية الإضبارة</oddHeader>
+    <oddFooter>&amp;C&amp;"Cairo,Regular"&amp;9DOS-37-2026-000004 | &amp;P / &amp;N</oddFooter>
   </headerFooter>
   <drawing r:id="rId1"/>
 </worksheet>
@@ -1510,77 +1512,77 @@
   <dimension ref="A1:D8"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="11.80859375" customWidth="true" style="69"/>
-    <col min="2" max="2" width="23.76953125" customWidth="true" style="69"/>
-    <col min="3" max="3" width="28.5234375" customWidth="true" style="69"/>
-    <col min="4" max="4" width="23.76953125" customWidth="true" style="69"/>
+    <col min="1" max="1" width="11.80859375" customWidth="true" style="70"/>
+    <col min="2" max="2" width="23.76953125" customWidth="true" style="70"/>
+    <col min="3" max="3" width="28.5234375" customWidth="true" style="70"/>
+    <col min="4" max="4" width="23.76953125" customWidth="true" style="70"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" customHeight="1" ht="47">
-      <c r="A1" s="69"/>
+      <c r="A1" s="70"/>
     </row>
     <row r="2" spans="1:4" customHeight="1" ht="34">
-      <c r="A2" s="70" t="s">
+      <c r="A2" s="71" t="s">
+        <v>79</v>
+      </c>
+      <c r="B2" s="71"/>
+      <c r="C2" s="71"/>
+      <c r="D2" s="71"/>
+    </row>
+    <row r="3" spans="1:4" customHeight="1" ht="30">
+      <c r="A3" s="72" t="s">
+        <v>44</v>
+      </c>
+      <c r="B3" s="72"/>
+      <c r="C3" s="72" t="s">
+        <v>45</v>
+      </c>
+      <c r="D3" s="72"/>
+    </row>
+    <row r="4" spans="1:4" customHeight="1" ht="30">
+      <c r="A4" s="72" t="s">
+        <v>46</v>
+      </c>
+      <c r="B4" s="72"/>
+      <c r="C4" s="72" t="s">
+        <v>47</v>
+      </c>
+      <c r="D4" s="72"/>
+    </row>
+    <row r="5" spans="1:4" customHeight="1" ht="22">
+      <c r="A5" s="72" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="72"/>
+      <c r="C5" s="72"/>
+      <c r="D5" s="72"/>
+    </row>
+    <row r="6" spans="1:4" customHeight="1" ht="36">
+      <c r="A6" s="72" t="s">
         <v>80</v>
       </c>
-      <c r="B2" s="70"/>
-      <c r="C2" s="70"/>
-      <c r="D2" s="70"/>
-    </row>
-    <row r="3" spans="1:4" customHeight="1" ht="30">
-      <c r="A3" s="71" t="s">
-        <v>45</v>
-      </c>
-      <c r="B3" s="71"/>
-      <c r="C3" s="71" t="s">
-        <v>46</v>
-      </c>
-      <c r="D3" s="71"/>
-    </row>
-    <row r="4" spans="1:4" customHeight="1" ht="30">
-      <c r="A4" s="71" t="s">
-        <v>47</v>
-      </c>
-      <c r="B4" s="71"/>
-      <c r="C4" s="71" t="s">
-        <v>48</v>
-      </c>
-      <c r="D4" s="71"/>
-    </row>
-    <row r="5" spans="1:4" customHeight="1" ht="22">
-      <c r="A5" s="71" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="71"/>
-      <c r="C5" s="71"/>
-      <c r="D5" s="71"/>
-    </row>
-    <row r="6" spans="1:4" customHeight="1" ht="36">
-      <c r="A6" s="71" t="s">
+      <c r="B6" s="72"/>
+      <c r="C6" s="72"/>
+      <c r="D6" s="72"/>
+    </row>
+    <row r="7" spans="1:4" customHeight="1" ht="8">
+      <c r="A7" s="72"/>
+      <c r="B7" s="72"/>
+      <c r="C7" s="72"/>
+      <c r="D7" s="72"/>
+    </row>
+    <row r="8" spans="1:4" customHeight="1" ht="29">
+      <c r="A8" s="73" t="s">
+        <v>49</v>
+      </c>
+      <c r="B8" s="73" t="s">
+        <v>58</v>
+      </c>
+      <c r="C8" s="73" t="s">
         <v>81</v>
       </c>
-      <c r="B6" s="71"/>
-      <c r="C6" s="71"/>
-      <c r="D6" s="71"/>
-    </row>
-    <row r="7" spans="1:4" customHeight="1" ht="8">
-      <c r="A7" s="71"/>
-      <c r="B7" s="71"/>
-      <c r="C7" s="71"/>
-      <c r="D7" s="71"/>
-    </row>
-    <row r="8" spans="1:4" customHeight="1" ht="29">
-      <c r="A8" s="72" t="s">
-        <v>50</v>
-      </c>
-      <c r="B8" s="72" t="s">
-        <v>59</v>
-      </c>
-      <c r="C8" s="72" t="s">
+      <c r="D8" s="73" t="s">
         <v>82</v>
-      </c>
-      <c r="D8" s="72" t="s">
-        <v>83</v>
       </c>
     </row>
   </sheetData>
@@ -1595,10 +1597,11 @@
     <mergeCell ref="A6:D6"/>
   </mergeCells>
   <printOptions gridLines="false" gridLinesSet="true"/>
-  <pageMargins left="0.47" right="0.47" top="0.35" bottom="0.5" header="0.3" footer="0.2"/>
+  <pageMargins left="0.47" right="0.47" top="0.5" bottom="0.5" header="0.18" footer="0.2"/>
   <pageSetup paperSize="9" orientation="portrait" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver"/>
   <headerFooter differentOddEven="false" differentFirst="false" scaleWithDoc="true" alignWithMargins="true">
-    <oddFooter>&amp;"Cairo,Regular"&amp;9&amp;CDOS-19-2026-000004 | &amp;P / &amp;N</oddFooter>
+    <oddHeader>&amp;R&amp;"Cairo,Regular"&amp;9الأدوية المصروفة</oddHeader>
+    <oddFooter>&amp;C&amp;"Cairo,Regular"&amp;9DOS-37-2026-000004 | &amp;P / &amp;N</oddFooter>
   </headerFooter>
   <drawing r:id="rId1"/>
 </worksheet>
@@ -1613,77 +1616,77 @@
   <dimension ref="A1:D8"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="11.80859375" customWidth="true" style="73"/>
-    <col min="2" max="2" width="23.76953125" customWidth="true" style="73"/>
-    <col min="3" max="3" width="28.5234375" customWidth="true" style="73"/>
-    <col min="4" max="4" width="23.76953125" customWidth="true" style="73"/>
+    <col min="1" max="1" width="11.80859375" customWidth="true" style="74"/>
+    <col min="2" max="2" width="23.76953125" customWidth="true" style="74"/>
+    <col min="3" max="3" width="28.5234375" customWidth="true" style="74"/>
+    <col min="4" max="4" width="23.76953125" customWidth="true" style="74"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" customHeight="1" ht="47">
-      <c r="A1" s="73"/>
+      <c r="A1" s="74"/>
     </row>
     <row r="2" spans="1:4" customHeight="1" ht="34">
-      <c r="A2" s="74" t="s">
-        <v>84</v>
-      </c>
-      <c r="B2" s="74"/>
-      <c r="C2" s="74"/>
-      <c r="D2" s="74"/>
+      <c r="A2" s="75" t="s">
+        <v>83</v>
+      </c>
+      <c r="B2" s="75"/>
+      <c r="C2" s="75"/>
+      <c r="D2" s="75"/>
     </row>
     <row r="3" spans="1:4" customHeight="1" ht="30">
-      <c r="A3" s="75" t="s">
+      <c r="A3" s="76" t="s">
+        <v>44</v>
+      </c>
+      <c r="B3" s="76"/>
+      <c r="C3" s="76" t="s">
         <v>45</v>
       </c>
-      <c r="B3" s="75"/>
-      <c r="C3" s="75" t="s">
+      <c r="D3" s="76"/>
+    </row>
+    <row r="4" spans="1:4" customHeight="1" ht="30">
+      <c r="A4" s="76" t="s">
         <v>46</v>
       </c>
-      <c r="D3" s="75"/>
-    </row>
-    <row r="4" spans="1:4" customHeight="1" ht="30">
-      <c r="A4" s="75" t="s">
+      <c r="B4" s="76"/>
+      <c r="C4" s="76" t="s">
         <v>47</v>
       </c>
-      <c r="B4" s="75"/>
-      <c r="C4" s="75" t="s">
-        <v>48</v>
-      </c>
-      <c r="D4" s="75"/>
+      <c r="D4" s="76"/>
     </row>
     <row r="5" spans="1:4" customHeight="1" ht="22">
-      <c r="A5" s="75" t="s">
+      <c r="A5" s="76" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="75"/>
-      <c r="C5" s="75"/>
-      <c r="D5" s="75"/>
+      <c r="B5" s="76"/>
+      <c r="C5" s="76"/>
+      <c r="D5" s="76"/>
     </row>
     <row r="6" spans="1:4" customHeight="1" ht="36">
-      <c r="A6" s="75" t="s">
+      <c r="A6" s="76" t="s">
+        <v>80</v>
+      </c>
+      <c r="B6" s="76"/>
+      <c r="C6" s="76"/>
+      <c r="D6" s="76"/>
+    </row>
+    <row r="7" spans="1:4" customHeight="1" ht="8">
+      <c r="A7" s="76"/>
+      <c r="B7" s="76"/>
+      <c r="C7" s="76"/>
+      <c r="D7" s="76"/>
+    </row>
+    <row r="8" spans="1:4" customHeight="1" ht="29">
+      <c r="A8" s="77" t="s">
+        <v>49</v>
+      </c>
+      <c r="B8" s="77" t="s">
+        <v>58</v>
+      </c>
+      <c r="C8" s="77" t="s">
         <v>81</v>
       </c>
-      <c r="B6" s="75"/>
-      <c r="C6" s="75"/>
-      <c r="D6" s="75"/>
-    </row>
-    <row r="7" spans="1:4" customHeight="1" ht="8">
-      <c r="A7" s="75"/>
-      <c r="B7" s="75"/>
-      <c r="C7" s="75"/>
-      <c r="D7" s="75"/>
-    </row>
-    <row r="8" spans="1:4" customHeight="1" ht="29">
-      <c r="A8" s="76" t="s">
-        <v>50</v>
-      </c>
-      <c r="B8" s="76" t="s">
-        <v>59</v>
-      </c>
-      <c r="C8" s="76" t="s">
+      <c r="D8" s="77" t="s">
         <v>82</v>
-      </c>
-      <c r="D8" s="76" t="s">
-        <v>83</v>
       </c>
     </row>
   </sheetData>
@@ -1698,10 +1701,11 @@
     <mergeCell ref="A6:D6"/>
   </mergeCells>
   <printOptions gridLines="false" gridLinesSet="true"/>
-  <pageMargins left="0.47" right="0.47" top="0.35" bottom="0.5" header="0.3" footer="0.2"/>
+  <pageMargins left="0.47" right="0.47" top="0.5" bottom="0.5" header="0.18" footer="0.2"/>
   <pageSetup paperSize="9" orientation="portrait" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver"/>
   <headerFooter differentOddEven="false" differentFirst="false" scaleWithDoc="true" alignWithMargins="true">
-    <oddFooter>&amp;"Cairo,Regular"&amp;9&amp;CDOS-19-2026-000004 | &amp;P / &amp;N</oddFooter>
+    <oddHeader>&amp;R&amp;"Cairo,Regular"&amp;9الأدوية المعطاة</oddHeader>
+    <oddFooter>&amp;C&amp;"Cairo,Regular"&amp;9DOS-37-2026-000004 | &amp;P / &amp;N</oddFooter>
   </headerFooter>
   <drawing r:id="rId1"/>
 </worksheet>
@@ -1716,104 +1720,104 @@
   <dimension ref="A1:E9"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="11.80859375" customWidth="true" style="77"/>
-    <col min="2" max="2" width="33.47265625" customWidth="true" style="77"/>
-    <col min="3" max="3" width="27.89453125" customWidth="true" style="77"/>
-    <col min="4" max="4" width="27.89453125" customWidth="true" style="77"/>
-    <col min="5" max="5" width="27.89453125" customWidth="true" style="77"/>
+    <col min="1" max="1" width="11.80859375" customWidth="true" style="78"/>
+    <col min="2" max="2" width="33.47265625" customWidth="true" style="78"/>
+    <col min="3" max="3" width="27.89453125" customWidth="true" style="78"/>
+    <col min="4" max="4" width="27.89453125" customWidth="true" style="78"/>
+    <col min="5" max="5" width="27.89453125" customWidth="true" style="78"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" customHeight="1" ht="47">
-      <c r="A1" s="77"/>
+      <c r="A1" s="78"/>
     </row>
     <row r="2" spans="1:5" customHeight="1" ht="34">
-      <c r="A2" s="78" t="s">
+      <c r="A2" s="79" t="s">
+        <v>84</v>
+      </c>
+      <c r="B2" s="79"/>
+      <c r="C2" s="79"/>
+      <c r="D2" s="79"/>
+      <c r="E2" s="79"/>
+    </row>
+    <row r="3" spans="1:5" customHeight="1" ht="30">
+      <c r="A3" s="80" t="s">
+        <v>44</v>
+      </c>
+      <c r="B3" s="80"/>
+      <c r="C3" s="80" t="s">
+        <v>45</v>
+      </c>
+      <c r="D3" s="80"/>
+      <c r="E3" s="80"/>
+    </row>
+    <row r="4" spans="1:5" customHeight="1" ht="30">
+      <c r="A4" s="80" t="s">
+        <v>46</v>
+      </c>
+      <c r="B4" s="80"/>
+      <c r="C4" s="80" t="s">
+        <v>47</v>
+      </c>
+      <c r="D4" s="80"/>
+      <c r="E4" s="80"/>
+    </row>
+    <row r="5" spans="1:5" customHeight="1" ht="22">
+      <c r="A5" s="80" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="80"/>
+      <c r="C5" s="80"/>
+      <c r="D5" s="80"/>
+      <c r="E5" s="80"/>
+    </row>
+    <row r="6" spans="1:5" customHeight="1" ht="22">
+      <c r="A6" s="80" t="s">
         <v>85</v>
       </c>
-      <c r="B2" s="78"/>
-      <c r="C2" s="78"/>
-      <c r="D2" s="78"/>
-      <c r="E2" s="78"/>
-    </row>
-    <row r="3" spans="1:5" customHeight="1" ht="30">
-      <c r="A3" s="79" t="s">
-        <v>45</v>
-      </c>
-      <c r="B3" s="79"/>
-      <c r="C3" s="79" t="s">
-        <v>46</v>
-      </c>
-      <c r="D3" s="79"/>
-      <c r="E3" s="79"/>
-    </row>
-    <row r="4" spans="1:5" customHeight="1" ht="30">
-      <c r="A4" s="79" t="s">
-        <v>47</v>
-      </c>
-      <c r="B4" s="79"/>
-      <c r="C4" s="79" t="s">
-        <v>48</v>
-      </c>
-      <c r="D4" s="79"/>
-      <c r="E4" s="79"/>
-    </row>
-    <row r="5" spans="1:5" customHeight="1" ht="22">
-      <c r="A5" s="79" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="79"/>
-      <c r="C5" s="79"/>
-      <c r="D5" s="79"/>
-      <c r="E5" s="79"/>
-    </row>
-    <row r="6" spans="1:5" customHeight="1" ht="22">
-      <c r="A6" s="79" t="s">
+      <c r="B6" s="80"/>
+      <c r="C6" s="80"/>
+      <c r="D6" s="80"/>
+      <c r="E6" s="80"/>
+    </row>
+    <row r="7" spans="1:5" customHeight="1" ht="8">
+      <c r="A7" s="80"/>
+      <c r="B7" s="80"/>
+      <c r="C7" s="80"/>
+      <c r="D7" s="80"/>
+      <c r="E7" s="80"/>
+    </row>
+    <row r="8" spans="1:5" customHeight="1" ht="29">
+      <c r="A8" s="81" t="s">
+        <v>49</v>
+      </c>
+      <c r="B8" s="81" t="s">
         <v>86</v>
       </c>
-      <c r="B6" s="79"/>
-      <c r="C6" s="79"/>
-      <c r="D6" s="79"/>
-      <c r="E6" s="79"/>
-    </row>
-    <row r="7" spans="1:5" customHeight="1" ht="8">
-      <c r="A7" s="79"/>
-      <c r="B7" s="79"/>
-      <c r="C7" s="79"/>
-      <c r="D7" s="79"/>
-      <c r="E7" s="79"/>
-    </row>
-    <row r="8" spans="1:5" customHeight="1" ht="29">
-      <c r="A8" s="80" t="s">
-        <v>50</v>
-      </c>
-      <c r="B8" s="80" t="s">
+      <c r="C8" s="81" t="s">
         <v>87</v>
       </c>
-      <c r="C8" s="80" t="s">
+      <c r="D8" s="81" t="s">
         <v>88</v>
       </c>
-      <c r="D8" s="80" t="s">
+      <c r="E8" s="81" t="s">
         <v>89</v>
       </c>
-      <c r="E8" s="80" t="s">
+    </row>
+    <row r="9" spans="1:5" customHeight="1" ht="97">
+      <c r="A9" s="82" t="s">
+        <v>53</v>
+      </c>
+      <c r="B9" s="83" t="s">
         <v>90</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" customHeight="1" ht="97">
-      <c r="A9" s="81" t="s">
-        <v>54</v>
-      </c>
-      <c r="B9" s="82" t="s">
+      <c r="C9" s="83" t="s">
         <v>91</v>
       </c>
-      <c r="C9" s="82" t="s">
-        <v>92</v>
-      </c>
-      <c r="D9" s="83">
+      <c r="D9" s="84">
         <v>68</v>
       </c>
-      <c r="E9" s="82" t="s">
-        <v>93</v>
+      <c r="E9" s="85">
+        <v>46280.50528935185139</v>
       </c>
     </row>
   </sheetData>
@@ -1828,10 +1832,11 @@
     <mergeCell ref="A6:E6"/>
   </mergeCells>
   <printOptions gridLines="false" gridLinesSet="true"/>
-  <pageMargins left="0.47" right="0.47" top="0.35" bottom="0.5" header="0.3" footer="0.2"/>
+  <pageMargins left="0.47" right="0.47" top="0.5" bottom="0.5" header="0.18" footer="0.2"/>
   <pageSetup paperSize="9" orientation="portrait" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver"/>
   <headerFooter differentOddEven="false" differentFirst="false" scaleWithDoc="true" alignWithMargins="true">
-    <oddFooter>&amp;"Cairo,Regular"&amp;9&amp;CDOS-19-2026-000004 | &amp;P / &amp;N</oddFooter>
+    <oddHeader>&amp;R&amp;"Cairo,Regular"&amp;9بيانات المرفقات</oddHeader>
+    <oddFooter>&amp;C&amp;"Cairo,Regular"&amp;9DOS-37-2026-000004 | &amp;P / &amp;N</oddFooter>
   </headerFooter>
   <drawing r:id="rId1"/>
 </worksheet>
@@ -1846,157 +1851,157 @@
   <dimension ref="A1:B21"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="24.56640625" customWidth="true" style="6"/>
-    <col min="2" max="2" width="63.3046875" customWidth="true" style="6"/>
+    <col min="1" max="1" width="24.56640625" customWidth="true" style="7"/>
+    <col min="2" max="2" width="63.3046875" customWidth="true" style="7"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" customHeight="1" ht="47">
-      <c r="A1" s="6"/>
+      <c r="A1" s="7"/>
     </row>
     <row r="2" spans="1:2" customHeight="1" ht="34">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="B2" s="8"/>
+    </row>
+    <row r="3" spans="1:2" customHeight="1" ht="30">
+      <c r="A3" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="9"/>
+    </row>
+    <row r="4" spans="1:2" customHeight="1" ht="30">
+      <c r="A4" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="9"/>
+    </row>
+    <row r="5" spans="1:2" customHeight="1" ht="22">
+      <c r="A5" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="9"/>
+    </row>
+    <row r="6" spans="1:2" customHeight="1" ht="22">
+      <c r="A6" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" s="9"/>
+    </row>
+    <row r="7" spans="1:2" customHeight="1" ht="8">
+      <c r="A7" s="9"/>
+      <c r="B7" s="9"/>
+    </row>
+    <row r="8" spans="1:2" customHeight="1" ht="29">
+      <c r="A8" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="B8" s="10" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" customHeight="1" ht="27.25">
+      <c r="A9" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="B2" s="7"/>
-    </row>
-    <row r="3" spans="1:2" customHeight="1" ht="30">
-      <c r="A3" s="8" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="8"/>
-    </row>
-    <row r="4" spans="1:2" customHeight="1" ht="30">
-      <c r="A4" s="8" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4" s="8"/>
-    </row>
-    <row r="5" spans="1:2" customHeight="1" ht="22">
-      <c r="A5" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="8"/>
-    </row>
-    <row r="6" spans="1:2" customHeight="1" ht="22">
-      <c r="A6" s="8" t="s">
-        <v>4</v>
-      </c>
-      <c r="B6" s="8"/>
-    </row>
-    <row r="7" spans="1:2" customHeight="1" ht="8">
-      <c r="A7" s="8"/>
-      <c r="B7" s="8"/>
-    </row>
-    <row r="8" spans="1:2" customHeight="1" ht="29">
-      <c r="A8" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="B8" s="9" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" customHeight="1" ht="27.25">
-      <c r="A9" s="10" t="s">
+      <c r="B9" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="B9" s="10" t="s">
+    </row>
+    <row r="10" spans="1:2" customHeight="1" ht="27.25">
+      <c r="A10" s="12" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="10" spans="1:2" customHeight="1" ht="27.25">
-      <c r="A10" s="11" t="s">
+      <c r="B10" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B10" s="11" t="s">
+    </row>
+    <row r="11" spans="1:2" customHeight="1" ht="27.25">
+      <c r="A11" s="11" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="11" spans="1:2" customHeight="1" ht="27.25">
-      <c r="A11" s="10" t="s">
+      <c r="B11" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="B11" s="10" t="s">
+    </row>
+    <row r="12" spans="1:2" customHeight="1" ht="27.25">
+      <c r="A12" s="12" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="12" spans="1:2" customHeight="1" ht="27.25">
-      <c r="A12" s="11" t="s">
+      <c r="B12" s="12" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" customHeight="1" ht="27.25">
+      <c r="A13" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="B12" s="11" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" customHeight="1" ht="27.25">
-      <c r="A13" s="10" t="s">
+      <c r="B13" s="11" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" customHeight="1" ht="27.25">
+      <c r="A14" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="B13" s="10" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" customHeight="1" ht="27.25">
-      <c r="A14" s="11" t="s">
+      <c r="B14" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="B14" s="11" t="s">
+    </row>
+    <row r="15" spans="1:2" customHeight="1" ht="27.25">
+      <c r="A15" s="11" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="15" spans="1:2" customHeight="1" ht="27.25">
-      <c r="A15" s="10" t="s">
+      <c r="B15" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="B15" s="10" t="s">
+    </row>
+    <row r="16" spans="1:2" customHeight="1" ht="27.25">
+      <c r="A16" s="12" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="16" spans="1:2" customHeight="1" ht="27.25">
-      <c r="A16" s="11" t="s">
+      <c r="B16" s="12" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" customHeight="1" ht="27.25">
+      <c r="A17" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="B16" s="11" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" customHeight="1" ht="27.25">
-      <c r="A17" s="10" t="s">
+      <c r="B17" s="11" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" customHeight="1" ht="27.25">
+      <c r="A18" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="B17" s="10" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" customHeight="1" ht="27.25">
-      <c r="A18" s="11" t="s">
+      <c r="B18" s="12" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" customHeight="1" ht="27.25">
+      <c r="A19" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="B18" s="11" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" customHeight="1" ht="27.25">
-      <c r="A19" s="10" t="s">
+      <c r="B19" s="11" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" customHeight="1" ht="27.25">
+      <c r="A20" s="12" t="s">
         <v>35</v>
       </c>
-      <c r="B19" s="10" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" customHeight="1" ht="27.25">
-      <c r="A20" s="11" t="s">
+      <c r="B20" s="12" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" customHeight="1" ht="27.25">
+      <c r="A21" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="B20" s="11" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" customHeight="1" ht="27.25">
-      <c r="A21" s="10" t="s">
-        <v>37</v>
-      </c>
-      <c r="B21" s="10" t="s">
-        <v>29</v>
+      <c r="B21" s="11" t="s">
+        <v>28</v>
       </c>
     </row>
   </sheetData>
@@ -2009,10 +2014,11 @@
     <mergeCell ref="A6:B6"/>
   </mergeCells>
   <printOptions gridLines="false" gridLinesSet="true"/>
-  <pageMargins left="0.47" right="0.47" top="0.35" bottom="0.5" header="0.3" footer="0.2"/>
+  <pageMargins left="0.47" right="0.47" top="0.5" bottom="0.5" header="0.18" footer="0.2"/>
   <pageSetup paperSize="9" orientation="portrait" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver"/>
   <headerFooter differentOddEven="false" differentFirst="false" scaleWithDoc="true" alignWithMargins="true">
-    <oddFooter>&amp;"Cairo,Regular"&amp;9&amp;CDOS-19-2026-000004 | &amp;P / &amp;N</oddFooter>
+    <oddHeader>&amp;R&amp;"Cairo,Regular"&amp;9بيانات المريض الحالية</oddHeader>
+    <oddFooter>&amp;C&amp;"Cairo,Regular"&amp;9DOS-37-2026-000004 | &amp;P / &amp;N</oddFooter>
   </headerFooter>
   <drawing r:id="rId1"/>
 </worksheet>
@@ -2027,77 +2033,77 @@
   <dimension ref="A1:B11"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="24.56640625" customWidth="true" style="12"/>
-    <col min="2" max="2" width="63.3046875" customWidth="true" style="12"/>
+    <col min="1" max="1" width="24.56640625" customWidth="true" style="13"/>
+    <col min="2" max="2" width="63.3046875" customWidth="true" style="13"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" customHeight="1" ht="47">
-      <c r="A1" s="12"/>
+      <c r="A1" s="13"/>
     </row>
     <row r="2" spans="1:2" customHeight="1" ht="34">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="14" t="s">
+        <v>37</v>
+      </c>
+      <c r="B2" s="14"/>
+    </row>
+    <row r="3" spans="1:2" customHeight="1" ht="30">
+      <c r="A3" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="15"/>
+    </row>
+    <row r="4" spans="1:2" customHeight="1" ht="30">
+      <c r="A4" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="15"/>
+    </row>
+    <row r="5" spans="1:2" customHeight="1" ht="22">
+      <c r="A5" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="15"/>
+    </row>
+    <row r="6" spans="1:2" customHeight="1" ht="22">
+      <c r="A6" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" s="15"/>
+    </row>
+    <row r="7" spans="1:2" customHeight="1" ht="8">
+      <c r="A7" s="15"/>
+      <c r="B7" s="15"/>
+    </row>
+    <row r="8" spans="1:2" customHeight="1" ht="29">
+      <c r="A8" s="16" t="s">
+        <v>5</v>
+      </c>
+      <c r="B8" s="16" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" customHeight="1" ht="27.25">
+      <c r="A9" s="17" t="s">
         <v>38</v>
       </c>
-      <c r="B2" s="13"/>
-    </row>
-    <row r="3" spans="1:2" customHeight="1" ht="30">
-      <c r="A3" s="14" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="14"/>
-    </row>
-    <row r="4" spans="1:2" customHeight="1" ht="30">
-      <c r="A4" s="14" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4" s="14"/>
-    </row>
-    <row r="5" spans="1:2" customHeight="1" ht="22">
-      <c r="A5" s="14" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="14"/>
-    </row>
-    <row r="6" spans="1:2" customHeight="1" ht="22">
-      <c r="A6" s="14" t="s">
-        <v>4</v>
-      </c>
-      <c r="B6" s="14"/>
-    </row>
-    <row r="7" spans="1:2" customHeight="1" ht="8">
-      <c r="A7" s="14"/>
-      <c r="B7" s="14"/>
-    </row>
-    <row r="8" spans="1:2" customHeight="1" ht="29">
-      <c r="A8" s="15" t="s">
-        <v>5</v>
-      </c>
-      <c r="B8" s="15" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" customHeight="1" ht="27.25">
-      <c r="A9" s="16" t="s">
+      <c r="B9" s="17" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" customHeight="1" ht="27.25">
+      <c r="A10" s="18" t="s">
         <v>39</v>
       </c>
-      <c r="B9" s="16" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" customHeight="1" ht="27.25">
-      <c r="A10" s="17" t="s">
+      <c r="B10" s="18" t="s">
         <v>40</v>
       </c>
-      <c r="B10" s="17" t="s">
+    </row>
+    <row r="11" spans="1:2" customHeight="1" ht="27.25">
+      <c r="A11" s="17" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="11" spans="1:2" customHeight="1" ht="27.25">
-      <c r="A11" s="16" t="s">
+      <c r="B11" s="17" t="s">
         <v>42</v>
-      </c>
-      <c r="B11" s="16" t="s">
-        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -2110,10 +2116,11 @@
     <mergeCell ref="A6:B6"/>
   </mergeCells>
   <printOptions gridLines="false" gridLinesSet="true"/>
-  <pageMargins left="0.47" right="0.47" top="0.35" bottom="0.5" header="0.3" footer="0.2"/>
+  <pageMargins left="0.47" right="0.47" top="0.5" bottom="0.5" header="0.18" footer="0.2"/>
   <pageSetup paperSize="9" orientation="portrait" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver"/>
   <headerFooter differentOddEven="false" differentFirst="false" scaleWithDoc="true" alignWithMargins="true">
-    <oddFooter>&amp;"Cairo,Regular"&amp;9&amp;CDOS-19-2026-000004 | &amp;P / &amp;N</oddFooter>
+    <oddHeader>&amp;R&amp;"Cairo,Regular"&amp;9المعلومات الطبية الحالية</oddHeader>
+    <oddFooter>&amp;C&amp;"Cairo,Regular"&amp;9DOS-37-2026-000004 | &amp;P / &amp;N</oddFooter>
   </headerFooter>
   <drawing r:id="rId1"/>
 </worksheet>
@@ -2128,91 +2135,91 @@
   <dimension ref="A1:D9"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="11.80859375" customWidth="true" style="18"/>
-    <col min="2" max="2" width="25.3515625" customWidth="true" style="18"/>
-    <col min="3" max="3" width="25.3515625" customWidth="true" style="18"/>
-    <col min="4" max="4" width="25.3515625" customWidth="true" style="18"/>
+    <col min="1" max="1" width="11.80859375" customWidth="true" style="19"/>
+    <col min="2" max="2" width="25.3515625" customWidth="true" style="19"/>
+    <col min="3" max="3" width="25.3515625" customWidth="true" style="19"/>
+    <col min="4" max="4" width="25.3515625" customWidth="true" style="19"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" customHeight="1" ht="47">
-      <c r="A1" s="18"/>
+      <c r="A1" s="19"/>
     </row>
     <row r="2" spans="1:4" customHeight="1" ht="34">
-      <c r="A2" s="19" t="s">
+      <c r="A2" s="20" t="s">
+        <v>43</v>
+      </c>
+      <c r="B2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+    </row>
+    <row r="3" spans="1:4" customHeight="1" ht="30">
+      <c r="A3" s="21" t="s">
         <v>44</v>
       </c>
-      <c r="B2" s="19"/>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-    </row>
-    <row r="3" spans="1:4" customHeight="1" ht="30">
-      <c r="A3" s="20" t="s">
+      <c r="B3" s="21"/>
+      <c r="C3" s="21" t="s">
         <v>45</v>
       </c>
-      <c r="B3" s="20"/>
-      <c r="C3" s="20" t="s">
+      <c r="D3" s="21"/>
+    </row>
+    <row r="4" spans="1:4" customHeight="1" ht="30">
+      <c r="A4" s="21" t="s">
         <v>46</v>
       </c>
-      <c r="D3" s="20"/>
-    </row>
-    <row r="4" spans="1:4" customHeight="1" ht="30">
-      <c r="A4" s="20" t="s">
+      <c r="B4" s="21"/>
+      <c r="C4" s="21" t="s">
         <v>47</v>
       </c>
-      <c r="B4" s="20"/>
-      <c r="C4" s="20" t="s">
+      <c r="D4" s="21"/>
+    </row>
+    <row r="5" spans="1:4" customHeight="1" ht="22">
+      <c r="A5" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="21"/>
+      <c r="C5" s="21"/>
+      <c r="D5" s="21"/>
+    </row>
+    <row r="6" spans="1:4" customHeight="1" ht="22">
+      <c r="A6" s="21" t="s">
         <v>48</v>
       </c>
-      <c r="D4" s="20"/>
-    </row>
-    <row r="5" spans="1:4" customHeight="1" ht="22">
-      <c r="A5" s="20" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="20"/>
-      <c r="C5" s="20"/>
-      <c r="D5" s="20"/>
-    </row>
-    <row r="6" spans="1:4" customHeight="1" ht="22">
-      <c r="A6" s="20" t="s">
+      <c r="B6" s="21"/>
+      <c r="C6" s="21"/>
+      <c r="D6" s="21"/>
+    </row>
+    <row r="7" spans="1:4" customHeight="1" ht="8">
+      <c r="A7" s="21"/>
+      <c r="B7" s="21"/>
+      <c r="C7" s="21"/>
+      <c r="D7" s="21"/>
+    </row>
+    <row r="8" spans="1:4" customHeight="1" ht="29">
+      <c r="A8" s="22" t="s">
         <v>49</v>
       </c>
-      <c r="B6" s="20"/>
-      <c r="C6" s="20"/>
-      <c r="D6" s="20"/>
-    </row>
-    <row r="7" spans="1:4" customHeight="1" ht="8">
-      <c r="A7" s="20"/>
-      <c r="B7" s="20"/>
-      <c r="C7" s="20"/>
-      <c r="D7" s="20"/>
-    </row>
-    <row r="8" spans="1:4" customHeight="1" ht="29">
-      <c r="A8" s="21" t="s">
+      <c r="B8" s="22" t="s">
         <v>50</v>
       </c>
-      <c r="B8" s="21" t="s">
+      <c r="C8" s="22" t="s">
         <v>51</v>
       </c>
-      <c r="C8" s="21" t="s">
+      <c r="D8" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="D8" s="21" t="s">
+    </row>
+    <row r="9" spans="1:4" customHeight="1" ht="97">
+      <c r="A9" s="23" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" customHeight="1" ht="97">
-      <c r="A9" s="22" t="s">
+      <c r="B9" s="24">
+        <v>36952.0</v>
+      </c>
+      <c r="C9" s="25" t="s">
         <v>54</v>
       </c>
-      <c r="B9" s="23">
-        <v>36952.0</v>
-      </c>
-      <c r="C9" s="24" t="s">
+      <c r="D9" s="25" t="s">
         <v>55</v>
-      </c>
-      <c r="D9" s="24" t="s">
-        <v>56</v>
       </c>
     </row>
   </sheetData>
@@ -2227,10 +2234,11 @@
     <mergeCell ref="A6:D6"/>
   </mergeCells>
   <printOptions gridLines="false" gridLinesSet="true"/>
-  <pageMargins left="0.47" right="0.47" top="0.35" bottom="0.5" header="0.3" footer="0.2"/>
+  <pageMargins left="0.47" right="0.47" top="0.5" bottom="0.5" header="0.18" footer="0.2"/>
   <pageSetup paperSize="9" orientation="portrait" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver"/>
   <headerFooter differentOddEven="false" differentFirst="false" scaleWithDoc="true" alignWithMargins="true">
-    <oddFooter>&amp;"Cairo,Regular"&amp;9&amp;CDOS-19-2026-000004 | &amp;P / &amp;N</oddFooter>
+    <oddHeader>&amp;R&amp;"Cairo,Regular"&amp;9التسلسل الزمني للزيارات</oddHeader>
+    <oddFooter>&amp;C&amp;"Cairo,Regular"&amp;9DOS-37-2026-000004 | &amp;P / &amp;N</oddFooter>
   </headerFooter>
   <drawing r:id="rId1"/>
 </worksheet>
@@ -2245,114 +2253,114 @@
   <dimension ref="A1:F9"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="11.80859375" customWidth="true" style="25"/>
-    <col min="2" max="2" width="22.53125" customWidth="true" style="25"/>
-    <col min="3" max="3" width="27.03515625" customWidth="true" style="25"/>
-    <col min="4" max="4" width="22.53125" customWidth="true" style="25"/>
-    <col min="5" max="5" width="22.53125" customWidth="true" style="25"/>
-    <col min="6" max="6" width="22.53125" customWidth="true" style="25"/>
+    <col min="1" max="1" width="11.80859375" customWidth="true" style="26"/>
+    <col min="2" max="2" width="22.53125" customWidth="true" style="26"/>
+    <col min="3" max="3" width="27.03515625" customWidth="true" style="26"/>
+    <col min="4" max="4" width="22.53125" customWidth="true" style="26"/>
+    <col min="5" max="5" width="22.53125" customWidth="true" style="26"/>
+    <col min="6" max="6" width="22.53125" customWidth="true" style="26"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" customHeight="1" ht="47">
-      <c r="A1" s="25"/>
+      <c r="A1" s="26"/>
     </row>
     <row r="2" spans="1:6" customHeight="1" ht="34">
-      <c r="A2" s="26" t="s">
+      <c r="A2" s="27" t="s">
+        <v>56</v>
+      </c>
+      <c r="B2" s="27"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="27"/>
+      <c r="F2" s="27"/>
+    </row>
+    <row r="3" spans="1:6" customHeight="1" ht="30">
+      <c r="A3" s="28" t="s">
+        <v>44</v>
+      </c>
+      <c r="B3" s="28"/>
+      <c r="C3" s="28"/>
+      <c r="D3" s="28" t="s">
+        <v>45</v>
+      </c>
+      <c r="E3" s="28"/>
+      <c r="F3" s="28"/>
+    </row>
+    <row r="4" spans="1:6" customHeight="1" ht="30">
+      <c r="A4" s="28" t="s">
+        <v>46</v>
+      </c>
+      <c r="B4" s="28"/>
+      <c r="C4" s="28"/>
+      <c r="D4" s="28" t="s">
+        <v>47</v>
+      </c>
+      <c r="E4" s="28"/>
+      <c r="F4" s="28"/>
+    </row>
+    <row r="5" spans="1:6" customHeight="1" ht="22">
+      <c r="A5" s="28" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="28"/>
+      <c r="C5" s="28"/>
+      <c r="D5" s="28"/>
+      <c r="E5" s="28"/>
+      <c r="F5" s="28"/>
+    </row>
+    <row r="6" spans="1:6" customHeight="1" ht="22">
+      <c r="A6" s="28" t="s">
         <v>57</v>
       </c>
-      <c r="B2" s="26"/>
-      <c r="C2" s="26"/>
-      <c r="D2" s="26"/>
-      <c r="E2" s="26"/>
-      <c r="F2" s="26"/>
-    </row>
-    <row r="3" spans="1:6" customHeight="1" ht="30">
-      <c r="A3" s="27" t="s">
-        <v>45</v>
-      </c>
-      <c r="B3" s="27"/>
-      <c r="C3" s="27"/>
-      <c r="D3" s="27" t="s">
-        <v>46</v>
-      </c>
-      <c r="E3" s="27"/>
-      <c r="F3" s="27"/>
-    </row>
-    <row r="4" spans="1:6" customHeight="1" ht="30">
-      <c r="A4" s="27" t="s">
-        <v>47</v>
-      </c>
-      <c r="B4" s="27"/>
-      <c r="C4" s="27"/>
-      <c r="D4" s="27" t="s">
-        <v>48</v>
-      </c>
-      <c r="E4" s="27"/>
-      <c r="F4" s="27"/>
-    </row>
-    <row r="5" spans="1:6" customHeight="1" ht="22">
-      <c r="A5" s="27" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="27"/>
-      <c r="C5" s="27"/>
-      <c r="D5" s="27"/>
-      <c r="E5" s="27"/>
-      <c r="F5" s="27"/>
-    </row>
-    <row r="6" spans="1:6" customHeight="1" ht="22">
-      <c r="A6" s="27" t="s">
+      <c r="B6" s="28"/>
+      <c r="C6" s="28"/>
+      <c r="D6" s="28"/>
+      <c r="E6" s="28"/>
+      <c r="F6" s="28"/>
+    </row>
+    <row r="7" spans="1:6" customHeight="1" ht="8">
+      <c r="A7" s="28"/>
+      <c r="B7" s="28"/>
+      <c r="C7" s="28"/>
+      <c r="D7" s="28"/>
+      <c r="E7" s="28"/>
+      <c r="F7" s="28"/>
+    </row>
+    <row r="8" spans="1:6" customHeight="1" ht="29">
+      <c r="A8" s="29" t="s">
+        <v>49</v>
+      </c>
+      <c r="B8" s="29" t="s">
         <v>58</v>
       </c>
-      <c r="B6" s="27"/>
-      <c r="C6" s="27"/>
-      <c r="D6" s="27"/>
-      <c r="E6" s="27"/>
-      <c r="F6" s="27"/>
-    </row>
-    <row r="7" spans="1:6" customHeight="1" ht="8">
-      <c r="A7" s="27"/>
-      <c r="B7" s="27"/>
-      <c r="C7" s="27"/>
-      <c r="D7" s="27"/>
-      <c r="E7" s="27"/>
-      <c r="F7" s="27"/>
-    </row>
-    <row r="8" spans="1:6" customHeight="1" ht="29">
-      <c r="A8" s="28" t="s">
-        <v>50</v>
-      </c>
-      <c r="B8" s="28" t="s">
+      <c r="C8" s="29" t="s">
+        <v>5</v>
+      </c>
+      <c r="D8" s="29" t="s">
         <v>59</v>
       </c>
-      <c r="C8" s="28" t="s">
-        <v>5</v>
-      </c>
-      <c r="D8" s="28" t="s">
+      <c r="E8" s="29" t="s">
         <v>60</v>
       </c>
-      <c r="E8" s="28" t="s">
+      <c r="F8" s="29" t="s">
         <v>61</v>
       </c>
-      <c r="F8" s="28" t="s">
+    </row>
+    <row r="9" spans="1:6" customHeight="1" ht="97">
+      <c r="A9" s="30" t="s">
+        <v>53</v>
+      </c>
+      <c r="B9" s="31"/>
+      <c r="C9" s="32" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" customHeight="1" ht="97">
-      <c r="A9" s="29" t="s">
-        <v>54</v>
-      </c>
-      <c r="B9" s="30"/>
-      <c r="C9" s="31" t="s">
+      <c r="D9" s="32" t="s">
         <v>63</v>
       </c>
-      <c r="D9" s="31" t="s">
+      <c r="E9" s="32" t="s">
         <v>64</v>
       </c>
-      <c r="E9" s="31" t="s">
-        <v>65</v>
-      </c>
-      <c r="F9" s="31"/>
+      <c r="F9" s="32"/>
     </row>
   </sheetData>
   <autoFilter ref="A8:F9"/>
@@ -2366,10 +2374,11 @@
     <mergeCell ref="A6:F6"/>
   </mergeCells>
   <printOptions gridLines="false" gridLinesSet="true"/>
-  <pageMargins left="0.47" right="0.47" top="0.35" bottom="0.5" header="0.3" footer="0.2"/>
+  <pageMargins left="0.47" right="0.47" top="0.5" bottom="0.5" header="0.18" footer="0.2"/>
   <pageSetup paperSize="9" orientation="portrait" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver"/>
   <headerFooter differentOddEven="false" differentFirst="false" scaleWithDoc="true" alignWithMargins="true">
-    <oddFooter>&amp;"Cairo,Regular"&amp;9&amp;CDOS-19-2026-000004 | &amp;P / &amp;N</oddFooter>
+    <oddHeader>&amp;R&amp;"Cairo,Regular"&amp;9التشخيصات</oddHeader>
+    <oddFooter>&amp;C&amp;"Cairo,Regular"&amp;9DOS-37-2026-000004 | &amp;P / &amp;N</oddFooter>
   </headerFooter>
   <drawing r:id="rId1"/>
 </worksheet>
@@ -2384,137 +2393,137 @@
   <dimension ref="A1:F10"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="11.80859375" customWidth="true" style="32"/>
-    <col min="2" max="2" width="22.53125" customWidth="true" style="32"/>
-    <col min="3" max="3" width="27.03515625" customWidth="true" style="32"/>
-    <col min="4" max="4" width="22.53125" customWidth="true" style="32"/>
-    <col min="5" max="5" width="22.53125" customWidth="true" style="32"/>
-    <col min="6" max="6" width="22.53125" customWidth="true" style="32"/>
+    <col min="1" max="1" width="11.80859375" customWidth="true" style="33"/>
+    <col min="2" max="2" width="22.53125" customWidth="true" style="33"/>
+    <col min="3" max="3" width="27.03515625" customWidth="true" style="33"/>
+    <col min="4" max="4" width="22.53125" customWidth="true" style="33"/>
+    <col min="5" max="5" width="22.53125" customWidth="true" style="33"/>
+    <col min="6" max="6" width="22.53125" customWidth="true" style="33"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" customHeight="1" ht="47">
-      <c r="A1" s="32"/>
+      <c r="A1" s="33"/>
     </row>
     <row r="2" spans="1:6" customHeight="1" ht="34">
-      <c r="A2" s="33" t="s">
+      <c r="A2" s="34" t="s">
+        <v>65</v>
+      </c>
+      <c r="B2" s="34"/>
+      <c r="C2" s="34"/>
+      <c r="D2" s="34"/>
+      <c r="E2" s="34"/>
+      <c r="F2" s="34"/>
+    </row>
+    <row r="3" spans="1:6" customHeight="1" ht="30">
+      <c r="A3" s="35" t="s">
+        <v>44</v>
+      </c>
+      <c r="B3" s="35"/>
+      <c r="C3" s="35"/>
+      <c r="D3" s="35" t="s">
+        <v>45</v>
+      </c>
+      <c r="E3" s="35"/>
+      <c r="F3" s="35"/>
+    </row>
+    <row r="4" spans="1:6" customHeight="1" ht="30">
+      <c r="A4" s="35" t="s">
+        <v>46</v>
+      </c>
+      <c r="B4" s="35"/>
+      <c r="C4" s="35"/>
+      <c r="D4" s="35" t="s">
+        <v>47</v>
+      </c>
+      <c r="E4" s="35"/>
+      <c r="F4" s="35"/>
+    </row>
+    <row r="5" spans="1:6" customHeight="1" ht="22">
+      <c r="A5" s="35" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="35"/>
+      <c r="C5" s="35"/>
+      <c r="D5" s="35"/>
+      <c r="E5" s="35"/>
+      <c r="F5" s="35"/>
+    </row>
+    <row r="6" spans="1:6" customHeight="1" ht="22">
+      <c r="A6" s="35" t="s">
+        <v>57</v>
+      </c>
+      <c r="B6" s="35"/>
+      <c r="C6" s="35"/>
+      <c r="D6" s="35"/>
+      <c r="E6" s="35"/>
+      <c r="F6" s="35"/>
+    </row>
+    <row r="7" spans="1:6" customHeight="1" ht="8">
+      <c r="A7" s="35"/>
+      <c r="B7" s="35"/>
+      <c r="C7" s="35"/>
+      <c r="D7" s="35"/>
+      <c r="E7" s="35"/>
+      <c r="F7" s="35"/>
+    </row>
+    <row r="8" spans="1:6" customHeight="1" ht="29">
+      <c r="A8" s="36" t="s">
+        <v>49</v>
+      </c>
+      <c r="B8" s="36" t="s">
+        <v>58</v>
+      </c>
+      <c r="C8" s="36" t="s">
+        <v>5</v>
+      </c>
+      <c r="D8" s="36" t="s">
+        <v>59</v>
+      </c>
+      <c r="E8" s="36" t="s">
+        <v>60</v>
+      </c>
+      <c r="F8" s="36" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" customHeight="1" ht="97">
+      <c r="A9" s="37" t="s">
+        <v>53</v>
+      </c>
+      <c r="B9" s="38">
+        <v>36952.0</v>
+      </c>
+      <c r="C9" s="39" t="s">
         <v>66</v>
       </c>
-      <c r="B2" s="33"/>
-      <c r="C2" s="33"/>
-      <c r="D2" s="33"/>
-      <c r="E2" s="33"/>
-      <c r="F2" s="33"/>
-    </row>
-    <row r="3" spans="1:6" customHeight="1" ht="30">
-      <c r="A3" s="34" t="s">
-        <v>45</v>
-      </c>
-      <c r="B3" s="34"/>
-      <c r="C3" s="34"/>
-      <c r="D3" s="34" t="s">
-        <v>46</v>
-      </c>
-      <c r="E3" s="34"/>
-      <c r="F3" s="34"/>
-    </row>
-    <row r="4" spans="1:6" customHeight="1" ht="30">
-      <c r="A4" s="34" t="s">
-        <v>47</v>
-      </c>
-      <c r="B4" s="34"/>
-      <c r="C4" s="34"/>
-      <c r="D4" s="34" t="s">
-        <v>48</v>
-      </c>
-      <c r="E4" s="34"/>
-      <c r="F4" s="34"/>
-    </row>
-    <row r="5" spans="1:6" customHeight="1" ht="22">
-      <c r="A5" s="34" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="34"/>
-      <c r="C5" s="34"/>
-      <c r="D5" s="34"/>
-      <c r="E5" s="34"/>
-      <c r="F5" s="34"/>
-    </row>
-    <row r="6" spans="1:6" customHeight="1" ht="22">
-      <c r="A6" s="34" t="s">
-        <v>58</v>
-      </c>
-      <c r="B6" s="34"/>
-      <c r="C6" s="34"/>
-      <c r="D6" s="34"/>
-      <c r="E6" s="34"/>
-      <c r="F6" s="34"/>
-    </row>
-    <row r="7" spans="1:6" customHeight="1" ht="8">
-      <c r="A7" s="34"/>
-      <c r="B7" s="34"/>
-      <c r="C7" s="34"/>
-      <c r="D7" s="34"/>
-      <c r="E7" s="34"/>
-      <c r="F7" s="34"/>
-    </row>
-    <row r="8" spans="1:6" customHeight="1" ht="29">
-      <c r="A8" s="35" t="s">
-        <v>50</v>
-      </c>
-      <c r="B8" s="35" t="s">
-        <v>59</v>
-      </c>
-      <c r="C8" s="35" t="s">
-        <v>5</v>
-      </c>
-      <c r="D8" s="35" t="s">
-        <v>60</v>
-      </c>
-      <c r="E8" s="35" t="s">
-        <v>61</v>
-      </c>
-      <c r="F8" s="35" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" customHeight="1" ht="97">
-      <c r="A9" s="36" t="s">
-        <v>54</v>
-      </c>
-      <c r="B9" s="37">
+      <c r="D9" s="39" t="s">
+        <v>63</v>
+      </c>
+      <c r="E9" s="39" t="s">
+        <v>64</v>
+      </c>
+      <c r="F9" s="39" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" customHeight="1" ht="97">
+      <c r="A10" s="40" t="s">
+        <v>53</v>
+      </c>
+      <c r="B10" s="41">
         <v>36952.0</v>
       </c>
-      <c r="C9" s="38" t="s">
+      <c r="C10" s="42" t="s">
+        <v>66</v>
+      </c>
+      <c r="D10" s="42" t="s">
+        <v>63</v>
+      </c>
+      <c r="E10" s="42" t="s">
+        <v>64</v>
+      </c>
+      <c r="F10" s="42" t="s">
         <v>67</v>
-      </c>
-      <c r="D9" s="38" t="s">
-        <v>64</v>
-      </c>
-      <c r="E9" s="38" t="s">
-        <v>65</v>
-      </c>
-      <c r="F9" s="38" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" customHeight="1" ht="97">
-      <c r="A10" s="39" t="s">
-        <v>54</v>
-      </c>
-      <c r="B10" s="40">
-        <v>36952.0</v>
-      </c>
-      <c r="C10" s="41" t="s">
-        <v>67</v>
-      </c>
-      <c r="D10" s="41" t="s">
-        <v>64</v>
-      </c>
-      <c r="E10" s="41" t="s">
-        <v>65</v>
-      </c>
-      <c r="F10" s="41" t="s">
-        <v>68</v>
       </c>
     </row>
   </sheetData>
@@ -2529,10 +2538,11 @@
     <mergeCell ref="A6:F6"/>
   </mergeCells>
   <printOptions gridLines="false" gridLinesSet="true"/>
-  <pageMargins left="0.47" right="0.47" top="0.35" bottom="0.5" header="0.3" footer="0.2"/>
+  <pageMargins left="0.47" right="0.47" top="0.5" bottom="0.5" header="0.18" footer="0.2"/>
   <pageSetup paperSize="9" orientation="portrait" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver"/>
   <headerFooter differentOddEven="false" differentFirst="false" scaleWithDoc="true" alignWithMargins="true">
-    <oddFooter>&amp;"Cairo,Regular"&amp;9&amp;CDOS-19-2026-000004 | &amp;P / &amp;N</oddFooter>
+    <oddHeader>&amp;R&amp;"Cairo,Regular"&amp;9الخدمات</oddHeader>
+    <oddFooter>&amp;C&amp;"Cairo,Regular"&amp;9DOS-37-2026-000004 | &amp;P / &amp;N</oddFooter>
   </headerFooter>
   <drawing r:id="rId1"/>
 </worksheet>
@@ -2547,137 +2557,137 @@
   <dimension ref="A1:F10"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="11.80859375" customWidth="true" style="42"/>
-    <col min="2" max="2" width="22.53125" customWidth="true" style="42"/>
-    <col min="3" max="3" width="27.03515625" customWidth="true" style="42"/>
-    <col min="4" max="4" width="22.53125" customWidth="true" style="42"/>
-    <col min="5" max="5" width="22.53125" customWidth="true" style="42"/>
-    <col min="6" max="6" width="22.53125" customWidth="true" style="42"/>
+    <col min="1" max="1" width="11.80859375" customWidth="true" style="43"/>
+    <col min="2" max="2" width="22.53125" customWidth="true" style="43"/>
+    <col min="3" max="3" width="27.03515625" customWidth="true" style="43"/>
+    <col min="4" max="4" width="22.53125" customWidth="true" style="43"/>
+    <col min="5" max="5" width="22.53125" customWidth="true" style="43"/>
+    <col min="6" max="6" width="22.53125" customWidth="true" style="43"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" customHeight="1" ht="47">
-      <c r="A1" s="42"/>
+      <c r="A1" s="43"/>
     </row>
     <row r="2" spans="1:6" customHeight="1" ht="34">
-      <c r="A2" s="43" t="s">
+      <c r="A2" s="44" t="s">
+        <v>68</v>
+      </c>
+      <c r="B2" s="44"/>
+      <c r="C2" s="44"/>
+      <c r="D2" s="44"/>
+      <c r="E2" s="44"/>
+      <c r="F2" s="44"/>
+    </row>
+    <row r="3" spans="1:6" customHeight="1" ht="30">
+      <c r="A3" s="45" t="s">
+        <v>44</v>
+      </c>
+      <c r="B3" s="45"/>
+      <c r="C3" s="45"/>
+      <c r="D3" s="45" t="s">
+        <v>45</v>
+      </c>
+      <c r="E3" s="45"/>
+      <c r="F3" s="45"/>
+    </row>
+    <row r="4" spans="1:6" customHeight="1" ht="30">
+      <c r="A4" s="45" t="s">
+        <v>46</v>
+      </c>
+      <c r="B4" s="45"/>
+      <c r="C4" s="45"/>
+      <c r="D4" s="45" t="s">
+        <v>47</v>
+      </c>
+      <c r="E4" s="45"/>
+      <c r="F4" s="45"/>
+    </row>
+    <row r="5" spans="1:6" customHeight="1" ht="22">
+      <c r="A5" s="45" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="45"/>
+      <c r="C5" s="45"/>
+      <c r="D5" s="45"/>
+      <c r="E5" s="45"/>
+      <c r="F5" s="45"/>
+    </row>
+    <row r="6" spans="1:6" customHeight="1" ht="22">
+      <c r="A6" s="45" t="s">
+        <v>57</v>
+      </c>
+      <c r="B6" s="45"/>
+      <c r="C6" s="45"/>
+      <c r="D6" s="45"/>
+      <c r="E6" s="45"/>
+      <c r="F6" s="45"/>
+    </row>
+    <row r="7" spans="1:6" customHeight="1" ht="8">
+      <c r="A7" s="45"/>
+      <c r="B7" s="45"/>
+      <c r="C7" s="45"/>
+      <c r="D7" s="45"/>
+      <c r="E7" s="45"/>
+      <c r="F7" s="45"/>
+    </row>
+    <row r="8" spans="1:6" customHeight="1" ht="29">
+      <c r="A8" s="46" t="s">
+        <v>49</v>
+      </c>
+      <c r="B8" s="46" t="s">
+        <v>58</v>
+      </c>
+      <c r="C8" s="46" t="s">
+        <v>5</v>
+      </c>
+      <c r="D8" s="46" t="s">
+        <v>59</v>
+      </c>
+      <c r="E8" s="46" t="s">
+        <v>60</v>
+      </c>
+      <c r="F8" s="46" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" customHeight="1" ht="97">
+      <c r="A9" s="47" t="s">
+        <v>53</v>
+      </c>
+      <c r="B9" s="48">
+        <v>36952.0</v>
+      </c>
+      <c r="C9" s="49" t="s">
         <v>69</v>
       </c>
-      <c r="B2" s="43"/>
-      <c r="C2" s="43"/>
-      <c r="D2" s="43"/>
-      <c r="E2" s="43"/>
-      <c r="F2" s="43"/>
-    </row>
-    <row r="3" spans="1:6" customHeight="1" ht="30">
-      <c r="A3" s="44" t="s">
-        <v>45</v>
-      </c>
-      <c r="B3" s="44"/>
-      <c r="C3" s="44"/>
-      <c r="D3" s="44" t="s">
-        <v>46</v>
-      </c>
-      <c r="E3" s="44"/>
-      <c r="F3" s="44"/>
-    </row>
-    <row r="4" spans="1:6" customHeight="1" ht="30">
-      <c r="A4" s="44" t="s">
-        <v>47</v>
-      </c>
-      <c r="B4" s="44"/>
-      <c r="C4" s="44"/>
-      <c r="D4" s="44" t="s">
-        <v>48</v>
-      </c>
-      <c r="E4" s="44"/>
-      <c r="F4" s="44"/>
-    </row>
-    <row r="5" spans="1:6" customHeight="1" ht="22">
-      <c r="A5" s="44" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="44"/>
-      <c r="C5" s="44"/>
-      <c r="D5" s="44"/>
-      <c r="E5" s="44"/>
-      <c r="F5" s="44"/>
-    </row>
-    <row r="6" spans="1:6" customHeight="1" ht="22">
-      <c r="A6" s="44" t="s">
-        <v>58</v>
-      </c>
-      <c r="B6" s="44"/>
-      <c r="C6" s="44"/>
-      <c r="D6" s="44"/>
-      <c r="E6" s="44"/>
-      <c r="F6" s="44"/>
-    </row>
-    <row r="7" spans="1:6" customHeight="1" ht="8">
-      <c r="A7" s="44"/>
-      <c r="B7" s="44"/>
-      <c r="C7" s="44"/>
-      <c r="D7" s="44"/>
-      <c r="E7" s="44"/>
-      <c r="F7" s="44"/>
-    </row>
-    <row r="8" spans="1:6" customHeight="1" ht="29">
-      <c r="A8" s="45" t="s">
-        <v>50</v>
-      </c>
-      <c r="B8" s="45" t="s">
-        <v>59</v>
-      </c>
-      <c r="C8" s="45" t="s">
-        <v>5</v>
-      </c>
-      <c r="D8" s="45" t="s">
-        <v>60</v>
-      </c>
-      <c r="E8" s="45" t="s">
-        <v>61</v>
-      </c>
-      <c r="F8" s="45" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" customHeight="1" ht="97">
-      <c r="A9" s="46" t="s">
-        <v>54</v>
-      </c>
-      <c r="B9" s="47">
+      <c r="D9" s="49" t="s">
+        <v>63</v>
+      </c>
+      <c r="E9" s="49" t="s">
+        <v>64</v>
+      </c>
+      <c r="F9" s="49" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" customHeight="1" ht="97">
+      <c r="A10" s="50" t="s">
+        <v>53</v>
+      </c>
+      <c r="B10" s="51">
         <v>36952.0</v>
       </c>
-      <c r="C9" s="48" t="s">
-        <v>70</v>
-      </c>
-      <c r="D9" s="48" t="s">
+      <c r="C10" s="52" t="s">
+        <v>69</v>
+      </c>
+      <c r="D10" s="52" t="s">
+        <v>63</v>
+      </c>
+      <c r="E10" s="52" t="s">
         <v>64</v>
       </c>
-      <c r="E9" s="48" t="s">
-        <v>65</v>
-      </c>
-      <c r="F9" s="48" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" customHeight="1" ht="97">
-      <c r="A10" s="49" t="s">
-        <v>54</v>
-      </c>
-      <c r="B10" s="50">
-        <v>36952.0</v>
-      </c>
-      <c r="C10" s="51" t="s">
-        <v>70</v>
-      </c>
-      <c r="D10" s="51" t="s">
-        <v>64</v>
-      </c>
-      <c r="E10" s="51" t="s">
-        <v>65</v>
-      </c>
-      <c r="F10" s="51" t="s">
-        <v>68</v>
+      <c r="F10" s="52" t="s">
+        <v>67</v>
       </c>
     </row>
   </sheetData>
@@ -2692,10 +2702,11 @@
     <mergeCell ref="A6:F6"/>
   </mergeCells>
   <printOptions gridLines="false" gridLinesSet="true"/>
-  <pageMargins left="0.47" right="0.47" top="0.35" bottom="0.5" header="0.3" footer="0.2"/>
+  <pageMargins left="0.47" right="0.47" top="0.5" bottom="0.5" header="0.18" footer="0.2"/>
   <pageSetup paperSize="9" orientation="portrait" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver"/>
   <headerFooter differentOddEven="false" differentFirst="false" scaleWithDoc="true" alignWithMargins="true">
-    <oddFooter>&amp;"Cairo,Regular"&amp;9&amp;CDOS-19-2026-000004 | &amp;P / &amp;N</oddFooter>
+    <oddHeader>&amp;R&amp;"Cairo,Regular"&amp;9الإجراءات</oddHeader>
+    <oddFooter>&amp;C&amp;"Cairo,Regular"&amp;9DOS-37-2026-000004 | &amp;P / &amp;N</oddFooter>
   </headerFooter>
   <drawing r:id="rId1"/>
 </worksheet>
@@ -2710,117 +2721,117 @@
   <dimension ref="A1:F9"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="11.80859375" customWidth="true" style="52"/>
-    <col min="2" max="2" width="22.53125" customWidth="true" style="52"/>
-    <col min="3" max="3" width="27.03515625" customWidth="true" style="52"/>
-    <col min="4" max="4" width="22.53125" customWidth="true" style="52"/>
-    <col min="5" max="5" width="22.53125" customWidth="true" style="52"/>
-    <col min="6" max="6" width="22.53125" customWidth="true" style="52"/>
+    <col min="1" max="1" width="11.80859375" customWidth="true" style="53"/>
+    <col min="2" max="2" width="22.53125" customWidth="true" style="53"/>
+    <col min="3" max="3" width="27.03515625" customWidth="true" style="53"/>
+    <col min="4" max="4" width="22.53125" customWidth="true" style="53"/>
+    <col min="5" max="5" width="22.53125" customWidth="true" style="53"/>
+    <col min="6" max="6" width="22.53125" customWidth="true" style="53"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" customHeight="1" ht="47">
-      <c r="A1" s="52"/>
+      <c r="A1" s="53"/>
     </row>
     <row r="2" spans="1:6" customHeight="1" ht="34">
-      <c r="A2" s="53" t="s">
+      <c r="A2" s="54" t="s">
+        <v>70</v>
+      </c>
+      <c r="B2" s="54"/>
+      <c r="C2" s="54"/>
+      <c r="D2" s="54"/>
+      <c r="E2" s="54"/>
+      <c r="F2" s="54"/>
+    </row>
+    <row r="3" spans="1:6" customHeight="1" ht="30">
+      <c r="A3" s="55" t="s">
+        <v>44</v>
+      </c>
+      <c r="B3" s="55"/>
+      <c r="C3" s="55"/>
+      <c r="D3" s="55" t="s">
+        <v>45</v>
+      </c>
+      <c r="E3" s="55"/>
+      <c r="F3" s="55"/>
+    </row>
+    <row r="4" spans="1:6" customHeight="1" ht="30">
+      <c r="A4" s="55" t="s">
+        <v>46</v>
+      </c>
+      <c r="B4" s="55"/>
+      <c r="C4" s="55"/>
+      <c r="D4" s="55" t="s">
+        <v>47</v>
+      </c>
+      <c r="E4" s="55"/>
+      <c r="F4" s="55"/>
+    </row>
+    <row r="5" spans="1:6" customHeight="1" ht="22">
+      <c r="A5" s="55" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="55"/>
+      <c r="C5" s="55"/>
+      <c r="D5" s="55"/>
+      <c r="E5" s="55"/>
+      <c r="F5" s="55"/>
+    </row>
+    <row r="6" spans="1:6" customHeight="1" ht="22">
+      <c r="A6" s="55" t="s">
+        <v>57</v>
+      </c>
+      <c r="B6" s="55"/>
+      <c r="C6" s="55"/>
+      <c r="D6" s="55"/>
+      <c r="E6" s="55"/>
+      <c r="F6" s="55"/>
+    </row>
+    <row r="7" spans="1:6" customHeight="1" ht="8">
+      <c r="A7" s="55"/>
+      <c r="B7" s="55"/>
+      <c r="C7" s="55"/>
+      <c r="D7" s="55"/>
+      <c r="E7" s="55"/>
+      <c r="F7" s="55"/>
+    </row>
+    <row r="8" spans="1:6" customHeight="1" ht="29">
+      <c r="A8" s="56" t="s">
+        <v>49</v>
+      </c>
+      <c r="B8" s="56" t="s">
+        <v>58</v>
+      </c>
+      <c r="C8" s="56" t="s">
+        <v>5</v>
+      </c>
+      <c r="D8" s="56" t="s">
+        <v>59</v>
+      </c>
+      <c r="E8" s="56" t="s">
+        <v>60</v>
+      </c>
+      <c r="F8" s="56" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" customHeight="1" ht="120.25">
+      <c r="A9" s="57" t="s">
+        <v>53</v>
+      </c>
+      <c r="B9" s="58">
+        <v>36952.0</v>
+      </c>
+      <c r="C9" s="59" t="s">
         <v>71</v>
       </c>
-      <c r="B2" s="53"/>
-      <c r="C2" s="53"/>
-      <c r="D2" s="53"/>
-      <c r="E2" s="53"/>
-      <c r="F2" s="53"/>
-    </row>
-    <row r="3" spans="1:6" customHeight="1" ht="30">
-      <c r="A3" s="54" t="s">
-        <v>45</v>
-      </c>
-      <c r="B3" s="54"/>
-      <c r="C3" s="54"/>
-      <c r="D3" s="54" t="s">
-        <v>46</v>
-      </c>
-      <c r="E3" s="54"/>
-      <c r="F3" s="54"/>
-    </row>
-    <row r="4" spans="1:6" customHeight="1" ht="30">
-      <c r="A4" s="54" t="s">
-        <v>47</v>
-      </c>
-      <c r="B4" s="54"/>
-      <c r="C4" s="54"/>
-      <c r="D4" s="54" t="s">
-        <v>48</v>
-      </c>
-      <c r="E4" s="54"/>
-      <c r="F4" s="54"/>
-    </row>
-    <row r="5" spans="1:6" customHeight="1" ht="22">
-      <c r="A5" s="54" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="54"/>
-      <c r="C5" s="54"/>
-      <c r="D5" s="54"/>
-      <c r="E5" s="54"/>
-      <c r="F5" s="54"/>
-    </row>
-    <row r="6" spans="1:6" customHeight="1" ht="22">
-      <c r="A6" s="54" t="s">
-        <v>58</v>
-      </c>
-      <c r="B6" s="54"/>
-      <c r="C6" s="54"/>
-      <c r="D6" s="54"/>
-      <c r="E6" s="54"/>
-      <c r="F6" s="54"/>
-    </row>
-    <row r="7" spans="1:6" customHeight="1" ht="8">
-      <c r="A7" s="54"/>
-      <c r="B7" s="54"/>
-      <c r="C7" s="54"/>
-      <c r="D7" s="54"/>
-      <c r="E7" s="54"/>
-      <c r="F7" s="54"/>
-    </row>
-    <row r="8" spans="1:6" customHeight="1" ht="29">
-      <c r="A8" s="55" t="s">
-        <v>50</v>
-      </c>
-      <c r="B8" s="55" t="s">
-        <v>59</v>
-      </c>
-      <c r="C8" s="55" t="s">
-        <v>5</v>
-      </c>
-      <c r="D8" s="55" t="s">
-        <v>60</v>
-      </c>
-      <c r="E8" s="55" t="s">
-        <v>61</v>
-      </c>
-      <c r="F8" s="55" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" customHeight="1" ht="120.25">
-      <c r="A9" s="56" t="s">
-        <v>54</v>
-      </c>
-      <c r="B9" s="57">
-        <v>36952.0</v>
-      </c>
-      <c r="C9" s="58" t="s">
+      <c r="D9" s="59" t="s">
+        <v>63</v>
+      </c>
+      <c r="E9" s="59" t="s">
+        <v>64</v>
+      </c>
+      <c r="F9" s="59" t="s">
         <v>72</v>
-      </c>
-      <c r="D9" s="58" t="s">
-        <v>64</v>
-      </c>
-      <c r="E9" s="58" t="s">
-        <v>65</v>
-      </c>
-      <c r="F9" s="58" t="s">
-        <v>73</v>
       </c>
     </row>
   </sheetData>
@@ -2835,10 +2846,11 @@
     <mergeCell ref="A6:F6"/>
   </mergeCells>
   <printOptions gridLines="false" gridLinesSet="true"/>
-  <pageMargins left="0.47" right="0.47" top="0.35" bottom="0.5" header="0.3" footer="0.2"/>
+  <pageMargins left="0.47" right="0.47" top="0.5" bottom="0.5" header="0.18" footer="0.2"/>
   <pageSetup paperSize="9" orientation="portrait" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver"/>
   <headerFooter differentOddEven="false" differentFirst="false" scaleWithDoc="true" alignWithMargins="true">
-    <oddFooter>&amp;"Cairo,Regular"&amp;9&amp;CDOS-19-2026-000004 | &amp;P / &amp;N</oddFooter>
+    <oddHeader>&amp;R&amp;"Cairo,Regular"&amp;9النتائج والإحالات الصادرة</oddHeader>
+    <oddFooter>&amp;C&amp;"Cairo,Regular"&amp;9DOS-37-2026-000004 | &amp;P / &amp;N</oddFooter>
   </headerFooter>
   <drawing r:id="rId1"/>
 </worksheet>
@@ -2853,137 +2865,137 @@
   <dimension ref="A1:F10"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="11.80859375" customWidth="true" style="59"/>
-    <col min="2" max="2" width="22.53125" customWidth="true" style="59"/>
-    <col min="3" max="3" width="27.03515625" customWidth="true" style="59"/>
-    <col min="4" max="4" width="22.53125" customWidth="true" style="59"/>
-    <col min="5" max="5" width="22.53125" customWidth="true" style="59"/>
-    <col min="6" max="6" width="22.53125" customWidth="true" style="59"/>
+    <col min="1" max="1" width="11.80859375" customWidth="true" style="60"/>
+    <col min="2" max="2" width="22.53125" customWidth="true" style="60"/>
+    <col min="3" max="3" width="27.03515625" customWidth="true" style="60"/>
+    <col min="4" max="4" width="22.53125" customWidth="true" style="60"/>
+    <col min="5" max="5" width="22.53125" customWidth="true" style="60"/>
+    <col min="6" max="6" width="22.53125" customWidth="true" style="60"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" customHeight="1" ht="47">
-      <c r="A1" s="59"/>
+      <c r="A1" s="60"/>
     </row>
     <row r="2" spans="1:6" customHeight="1" ht="34">
-      <c r="A2" s="60" t="s">
+      <c r="A2" s="61" t="s">
+        <v>73</v>
+      </c>
+      <c r="B2" s="61"/>
+      <c r="C2" s="61"/>
+      <c r="D2" s="61"/>
+      <c r="E2" s="61"/>
+      <c r="F2" s="61"/>
+    </row>
+    <row r="3" spans="1:6" customHeight="1" ht="30">
+      <c r="A3" s="62" t="s">
+        <v>44</v>
+      </c>
+      <c r="B3" s="62"/>
+      <c r="C3" s="62"/>
+      <c r="D3" s="62" t="s">
+        <v>45</v>
+      </c>
+      <c r="E3" s="62"/>
+      <c r="F3" s="62"/>
+    </row>
+    <row r="4" spans="1:6" customHeight="1" ht="30">
+      <c r="A4" s="62" t="s">
+        <v>46</v>
+      </c>
+      <c r="B4" s="62"/>
+      <c r="C4" s="62"/>
+      <c r="D4" s="62" t="s">
+        <v>47</v>
+      </c>
+      <c r="E4" s="62"/>
+      <c r="F4" s="62"/>
+    </row>
+    <row r="5" spans="1:6" customHeight="1" ht="22">
+      <c r="A5" s="62" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="62"/>
+      <c r="C5" s="62"/>
+      <c r="D5" s="62"/>
+      <c r="E5" s="62"/>
+      <c r="F5" s="62"/>
+    </row>
+    <row r="6" spans="1:6" customHeight="1" ht="22">
+      <c r="A6" s="62" t="s">
         <v>74</v>
       </c>
-      <c r="B2" s="60"/>
-      <c r="C2" s="60"/>
-      <c r="D2" s="60"/>
-      <c r="E2" s="60"/>
-      <c r="F2" s="60"/>
-    </row>
-    <row r="3" spans="1:6" customHeight="1" ht="30">
-      <c r="A3" s="61" t="s">
-        <v>45</v>
-      </c>
-      <c r="B3" s="61"/>
-      <c r="C3" s="61"/>
-      <c r="D3" s="61" t="s">
-        <v>46</v>
-      </c>
-      <c r="E3" s="61"/>
-      <c r="F3" s="61"/>
-    </row>
-    <row r="4" spans="1:6" customHeight="1" ht="30">
-      <c r="A4" s="61" t="s">
-        <v>47</v>
-      </c>
-      <c r="B4" s="61"/>
-      <c r="C4" s="61"/>
-      <c r="D4" s="61" t="s">
-        <v>48</v>
-      </c>
-      <c r="E4" s="61"/>
-      <c r="F4" s="61"/>
-    </row>
-    <row r="5" spans="1:6" customHeight="1" ht="22">
-      <c r="A5" s="61" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="61"/>
-      <c r="C5" s="61"/>
-      <c r="D5" s="61"/>
-      <c r="E5" s="61"/>
-      <c r="F5" s="61"/>
-    </row>
-    <row r="6" spans="1:6" customHeight="1" ht="22">
-      <c r="A6" s="61" t="s">
+      <c r="B6" s="62"/>
+      <c r="C6" s="62"/>
+      <c r="D6" s="62"/>
+      <c r="E6" s="62"/>
+      <c r="F6" s="62"/>
+    </row>
+    <row r="7" spans="1:6" customHeight="1" ht="8">
+      <c r="A7" s="62"/>
+      <c r="B7" s="62"/>
+      <c r="C7" s="62"/>
+      <c r="D7" s="62"/>
+      <c r="E7" s="62"/>
+      <c r="F7" s="62"/>
+    </row>
+    <row r="8" spans="1:6" customHeight="1" ht="29">
+      <c r="A8" s="63" t="s">
+        <v>49</v>
+      </c>
+      <c r="B8" s="63" t="s">
+        <v>58</v>
+      </c>
+      <c r="C8" s="63" t="s">
+        <v>5</v>
+      </c>
+      <c r="D8" s="63" t="s">
+        <v>59</v>
+      </c>
+      <c r="E8" s="63" t="s">
+        <v>60</v>
+      </c>
+      <c r="F8" s="63" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" customHeight="1" ht="97">
+      <c r="A9" s="64" t="s">
+        <v>53</v>
+      </c>
+      <c r="B9" s="65">
+        <v>36952.0</v>
+      </c>
+      <c r="C9" s="66" t="s">
         <v>75</v>
       </c>
-      <c r="B6" s="61"/>
-      <c r="C6" s="61"/>
-      <c r="D6" s="61"/>
-      <c r="E6" s="61"/>
-      <c r="F6" s="61"/>
-    </row>
-    <row r="7" spans="1:6" customHeight="1" ht="8">
-      <c r="A7" s="61"/>
-      <c r="B7" s="61"/>
-      <c r="C7" s="61"/>
-      <c r="D7" s="61"/>
-      <c r="E7" s="61"/>
-      <c r="F7" s="61"/>
-    </row>
-    <row r="8" spans="1:6" customHeight="1" ht="29">
-      <c r="A8" s="62" t="s">
-        <v>50</v>
-      </c>
-      <c r="B8" s="62" t="s">
-        <v>59</v>
-      </c>
-      <c r="C8" s="62" t="s">
-        <v>5</v>
-      </c>
-      <c r="D8" s="62" t="s">
-        <v>60</v>
-      </c>
-      <c r="E8" s="62" t="s">
-        <v>61</v>
-      </c>
-      <c r="F8" s="62" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" customHeight="1" ht="97">
-      <c r="A9" s="63" t="s">
-        <v>54</v>
-      </c>
-      <c r="B9" s="64">
+      <c r="D9" s="66" t="s">
+        <v>63</v>
+      </c>
+      <c r="E9" s="66" t="s">
+        <v>64</v>
+      </c>
+      <c r="F9" s="66" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" customHeight="1" ht="97">
+      <c r="A10" s="67" t="s">
+        <v>53</v>
+      </c>
+      <c r="B10" s="68">
         <v>36952.0</v>
       </c>
-      <c r="C9" s="65" t="s">
-        <v>76</v>
-      </c>
-      <c r="D9" s="65" t="s">
+      <c r="C10" s="69" t="s">
+        <v>77</v>
+      </c>
+      <c r="D10" s="69" t="s">
+        <v>63</v>
+      </c>
+      <c r="E10" s="69" t="s">
         <v>64</v>
       </c>
-      <c r="E9" s="65" t="s">
-        <v>65</v>
-      </c>
-      <c r="F9" s="65" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" customHeight="1" ht="97">
-      <c r="A10" s="66" t="s">
-        <v>54</v>
-      </c>
-      <c r="B10" s="67">
-        <v>36952.0</v>
-      </c>
-      <c r="C10" s="68" t="s">
+      <c r="F10" s="69" t="s">
         <v>78</v>
-      </c>
-      <c r="D10" s="68" t="s">
-        <v>64</v>
-      </c>
-      <c r="E10" s="68" t="s">
-        <v>65</v>
-      </c>
-      <c r="F10" s="68" t="s">
-        <v>79</v>
       </c>
     </row>
   </sheetData>
@@ -2998,10 +3010,11 @@
     <mergeCell ref="A6:F6"/>
   </mergeCells>
   <printOptions gridLines="false" gridLinesSet="true"/>
-  <pageMargins left="0.47" right="0.47" top="0.35" bottom="0.5" header="0.3" footer="0.2"/>
+  <pageMargins left="0.47" right="0.47" top="0.5" bottom="0.5" header="0.18" footer="0.2"/>
   <pageSetup paperSize="9" orientation="portrait" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver"/>
   <headerFooter differentOddEven="false" differentFirst="false" scaleWithDoc="true" alignWithMargins="true">
-    <oddFooter>&amp;"Cairo,Regular"&amp;9&amp;CDOS-19-2026-000004 | &amp;P / &amp;N</oddFooter>
+    <oddHeader>&amp;R&amp;"Cairo,Regular"&amp;9الأدوية الموصوفة</oddHeader>
+    <oddFooter>&amp;C&amp;"Cairo,Regular"&amp;9DOS-37-2026-000004 | &amp;P / &amp;N</oddFooter>
   </headerFooter>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>